<commit_message>
Deploying to main from @ pedalboard/pedalboard-display@aee31764f72741e6697704d457c2198dc5ab8179 🚀
</commit_message>
<xml_diff>
--- a/latest/BoM/Costs/pedalboard-display-bom.xlsx
+++ b/latest/BoM/Costs/pedalboard-display-bom.xlsx
@@ -484,7 +484,7 @@
     <t>KiCad Version:</t>
   </si>
   <si>
-    <t>8.0.6+1</t>
+    <t>9.0.1</t>
   </si>
   <si>
     <t>Component Groups:</t>
@@ -559,10 +559,10 @@
     <t>Created:</t>
   </si>
   <si>
-    <t>2024-12-24 11:54:47</t>
-  </si>
-  <si>
-    <t>KiCost® v1.1.19 + KiBot v1.8.2</t>
+    <t>2025-04-21 13:34:30</t>
+  </si>
+  <si>
+    <t>KiCost® v1.1.20 + KiBot v1.8.4</t>
   </si>
   <si>
     <t>Resistor</t>
@@ -961,10 +961,10 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>357600</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>297815</xdr:rowOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>16584</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>123779</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -991,7 +991,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="9396825" cy="5079365"/>
+          <a:ext cx="2378784" cy="1285829"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1013,10 +1013,10 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>3024600</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>107315</xdr:rowOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>16584</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>123779</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1043,7 +1043,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="9396825" cy="5079365"/>
+          <a:ext cx="2378784" cy="1285829"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1065,10 +1065,10 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>786225</xdr:colOff>
-      <xdr:row>13</xdr:row>
-      <xdr:rowOff>107315</xdr:rowOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>2378784</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>123779</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1095,7 +1095,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="9396825" cy="5079365"/>
+          <a:ext cx="2378784" cy="1285829"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1117,10 +1117,10 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>290925</xdr:colOff>
-      <xdr:row>25</xdr:row>
-      <xdr:rowOff>107315</xdr:rowOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>883359</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>123779</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1147,7 +1147,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="9396825" cy="5079365"/>
+          <a:ext cx="2378784" cy="1285829"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>

</xml_diff>